<commit_message>
To fix one file for update/register product
</commit_message>
<xml_diff>
--- a/api/storage/files/default_file/Padrão_Importação.xlsx
+++ b/api/storage/files/default_file/Padrão_Importação.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t xml:space="preserve">Nome produto</t>
   </si>
@@ -28,10 +28,13 @@
     <t xml:space="preserve">Preço de custo</t>
   </si>
   <si>
+    <t xml:space="preserve">Perce. De Lucro</t>
+  </si>
+  <si>
     <t xml:space="preserve">Preço de venda</t>
   </si>
   <si>
-    <t xml:space="preserve">Perce. De Lucro</t>
+    <t xml:space="preserve">Qtde</t>
   </si>
   <si>
     <t xml:space="preserve">CFOP</t>
@@ -51,7 +54,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0.00"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -72,6 +75,11 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -116,12 +124,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -252,11 +264,12 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16.74"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15.36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14.93"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -266,13 +279,13 @@
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="0" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
@@ -281,14 +294,14 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
+      <c r="B2" s="3"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>